<commit_message>
chore(quang): quan ly luu tru thu muc ai va cap nhat task tracking Hoan thanh (Tasks Q16, Q17)
</commit_message>
<xml_diff>
--- a/Group02_Task_List.xlsx
+++ b/Group02_Task_List.xlsx
@@ -607,7 +607,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -815,7 +814,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Sẵn sàng</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -888,7 +887,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="B12" s="15" t="inlineStr">
         <is>
@@ -4097,7 +4095,7 @@
       </c>
       <c r="I63" s="4" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J63" s="5" t="inlineStr">
@@ -4147,7 +4145,7 @@
       </c>
       <c r="I64" s="4" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J64" s="5" t="inlineStr">
@@ -4197,7 +4195,7 @@
       </c>
       <c r="I65" s="4" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J65" s="5" t="inlineStr">
@@ -4247,7 +4245,7 @@
       </c>
       <c r="I66" s="4" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J66" s="5" t="inlineStr">
@@ -4297,7 +4295,7 @@
       </c>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J67" s="5" t="inlineStr">
@@ -4347,7 +4345,7 @@
       </c>
       <c r="I68" s="4" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J68" s="5" t="inlineStr">
@@ -4397,7 +4395,7 @@
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J69" s="5" t="inlineStr">
@@ -4447,7 +4445,7 @@
       </c>
       <c r="I70" s="4" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J70" s="5" t="inlineStr">
@@ -4497,7 +4495,7 @@
       </c>
       <c r="I71" s="4" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J71" s="5" t="inlineStr">
@@ -4547,7 +4545,7 @@
       </c>
       <c r="I72" s="4" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J72" s="5" t="inlineStr">
@@ -4597,7 +4595,7 @@
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J73" s="5" t="inlineStr">
@@ -4647,7 +4645,7 @@
       </c>
       <c r="I74" s="4" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J74" s="5" t="inlineStr">
@@ -4697,7 +4695,7 @@
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J75" s="5" t="inlineStr">
@@ -4747,7 +4745,7 @@
       </c>
       <c r="I76" s="4" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J76" s="5" t="inlineStr">
@@ -4797,7 +4795,7 @@
       </c>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J77" s="5" t="inlineStr">
@@ -4847,7 +4845,7 @@
       </c>
       <c r="I78" s="4" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J78" s="5" t="inlineStr">
@@ -4897,7 +4895,7 @@
       </c>
       <c r="I79" s="4" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J79" s="5" t="inlineStr">

</xml_diff>